<commit_message>
fix(opay): scrub lastModifiedBy in xlsx redactor
Raw opay exports carry the template author's name in core props. The redactor kept it. The committed sample.xlsx is patched in place, since it is a trimmed copy and can't be regenerated.
</commit_message>
<xml_diff>
--- a/tests/opay/fixtures/sample.xlsx
+++ b/tests/opay/fixtures/sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="22060" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Wallet Account Transactions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Savings Account Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wallet Account Transactions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Savings Account Transactions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1179,7 +1179,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14" defaultRowHeight="15.2"/>
   <cols>
     <col width="21.0865384615385" customWidth="1" style="18" min="1" max="1"/>
@@ -2071,7 +2071,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="F2:H2"/>

</xml_diff>